<commit_message>
chore(import): add the email column to the downloadable sample template
Matches the new mappable email field — header + a filled example value.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/resources/templates/gamoryid-inventory-import-template.xlsx
+++ b/backend/resources/templates/gamoryid-inventory-import-template.xlsx
@@ -401,8 +401,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GamoryInventoryImport" displayName="GamoryInventoryImport" ref="A1:I2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="GamoryInventoryImport" displayName="GamoryInventoryImport" ref="A1:J2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="10">
     <x:tableColumn id="1" name="riot_id"/>
     <x:tableColumn id="2" name="username"/>
     <x:tableColumn id="3" name="password"/>
@@ -412,6 +412,7 @@
     <x:tableColumn id="7" name="cost"/>
     <x:tableColumn id="8" name="list_price"/>
     <x:tableColumn id="9" name="notes"/>
+    <x:tableColumn id="10" name="email"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -621,6 +622,7 @@
     <x:col min="7" max="7" width="15" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="15" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="35" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -651,6 +653,9 @@
       <x:c r="I1" s="22" t="str">
         <x:v>notes</x:v>
       </x:c>
+      <x:c r="J1" s="22" t="str">
+        <x:v>email</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="52" customHeight="1">
       <x:c r="A2" s="23" t="str">
@@ -679,6 +684,9 @@
       </x:c>
       <x:c r="I2" s="23" t="str">
         <x:v>ตัวอย่าง: ลูกค้ากำลังพิจารณา</x:v>
+      </x:c>
+      <x:c r="J2" s="23" t="str">
+        <x:v>example.user01@mail.test</x:v>
       </x:c>
     </x:row>
     <x:row r="3">

</xml_diff>